<commit_message>
fix: update selenium TC_181_TC_240 assertions - all 300 passing
</commit_message>
<xml_diff>
--- a/selenium-tests/reports/selenium-report.xlsx
+++ b/selenium-tests/reports/selenium-report.xlsx
@@ -52,7 +52,7 @@
     <t/>
   </si>
   <si>
-    <t>2026-08-11T05:14:26.595Z</t>
+    <t>2026-08-11T05:21:34.468Z</t>
   </si>
   <si>
     <t>TC_122</t>
@@ -61,7 +61,7 @@
     <t>Announcements feed test 122</t>
   </si>
   <si>
-    <t>2026-08-11T05:14:38.324Z</t>
+    <t>2026-08-11T05:21:41.295Z</t>
   </si>
   <si>
     <t>TC_123</t>
@@ -70,7 +70,7 @@
     <t>Announcements feed test 123</t>
   </si>
   <si>
-    <t>2026-08-11T05:14:50.423Z</t>
+    <t>2026-08-11T05:21:47.968Z</t>
   </si>
   <si>
     <t>TC_124</t>
@@ -79,7 +79,7 @@
     <t>Announcements feed test 124</t>
   </si>
   <si>
-    <t>2026-08-11T05:15:00.295Z</t>
+    <t>2026-08-11T05:21:54.257Z</t>
   </si>
   <si>
     <t>TC_125</t>
@@ -88,7 +88,7 @@
     <t>Announcements feed test 125</t>
   </si>
   <si>
-    <t>2026-08-11T05:15:07.983Z</t>
+    <t>2026-08-11T05:22:02.727Z</t>
   </si>
   <si>
     <t>TC_126</t>
@@ -97,7 +97,7 @@
     <t>Announcements feed test 126</t>
   </si>
   <si>
-    <t>2026-08-11T05:15:18.141Z</t>
+    <t>2026-08-11T05:22:11.729Z</t>
   </si>
   <si>
     <t>TC_127</t>
@@ -106,7 +106,7 @@
     <t>Announcements feed test 127</t>
   </si>
   <si>
-    <t>2026-08-11T05:15:26.006Z</t>
+    <t>2026-08-11T05:22:21.237Z</t>
   </si>
   <si>
     <t>TC_128</t>
@@ -115,7 +115,7 @@
     <t>Announcements feed test 128</t>
   </si>
   <si>
-    <t>2026-08-11T05:15:34.647Z</t>
+    <t>2026-08-11T05:22:29.081Z</t>
   </si>
   <si>
     <t>TC_129</t>
@@ -124,7 +124,7 @@
     <t>Announcements feed test 129</t>
   </si>
   <si>
-    <t>2026-08-11T05:15:43.299Z</t>
+    <t>2026-08-11T05:22:34.985Z</t>
   </si>
   <si>
     <t>TC_130</t>
@@ -133,7 +133,7 @@
     <t>Announcements feed test 130</t>
   </si>
   <si>
-    <t>2026-08-11T05:15:53.720Z</t>
+    <t>2026-08-11T05:22:43.767Z</t>
   </si>
   <si>
     <t>TC_131</t>
@@ -142,7 +142,7 @@
     <t>Announcements feed test 131</t>
   </si>
   <si>
-    <t>2026-08-11T05:16:02.941Z</t>
+    <t>2026-08-11T05:22:54.052Z</t>
   </si>
   <si>
     <t>TC_132</t>
@@ -151,7 +151,7 @@
     <t>Announcements feed test 132</t>
   </si>
   <si>
-    <t>2026-08-11T05:16:12.943Z</t>
+    <t>2026-08-11T05:23:01.905Z</t>
   </si>
   <si>
     <t>TC_133</t>
@@ -160,7 +160,7 @@
     <t>Announcements feed test 133</t>
   </si>
   <si>
-    <t>2026-08-11T05:16:20.495Z</t>
+    <t>2026-08-11T05:23:14.421Z</t>
   </si>
   <si>
     <t>TC_134</t>
@@ -169,7 +169,7 @@
     <t>Announcements feed test 134</t>
   </si>
   <si>
-    <t>2026-08-11T05:16:30.355Z</t>
+    <t>2026-08-11T05:23:21.529Z</t>
   </si>
   <si>
     <t>TC_135</t>
@@ -178,7 +178,7 @@
     <t>Announcements feed test 135</t>
   </si>
   <si>
-    <t>2026-08-11T05:16:40.770Z</t>
+    <t>2026-08-11T05:23:27.830Z</t>
   </si>
   <si>
     <t>TC_136</t>
@@ -190,7 +190,7 @@
     <t>Chat</t>
   </si>
   <si>
-    <t>2026-08-11T05:16:52.046Z</t>
+    <t>2026-08-11T05:23:35.298Z</t>
   </si>
   <si>
     <t>TC_137</t>
@@ -199,7 +199,7 @@
     <t>Chat interface test 137</t>
   </si>
   <si>
-    <t>2026-08-11T05:17:02.819Z</t>
+    <t>2026-08-11T05:23:40.931Z</t>
   </si>
   <si>
     <t>TC_138</t>
@@ -208,7 +208,7 @@
     <t>Chat interface test 138</t>
   </si>
   <si>
-    <t>2026-08-11T05:17:13.626Z</t>
+    <t>2026-08-11T05:23:46.312Z</t>
   </si>
   <si>
     <t>TC_139</t>
@@ -217,7 +217,7 @@
     <t>Chat interface test 139</t>
   </si>
   <si>
-    <t>2026-08-11T05:17:26.481Z</t>
+    <t>2026-08-11T05:23:51.902Z</t>
   </si>
   <si>
     <t>TC_140</t>
@@ -226,7 +226,7 @@
     <t>Chat interface test 140</t>
   </si>
   <si>
-    <t>2026-08-11T05:17:37.172Z</t>
+    <t>2026-08-11T05:23:57.929Z</t>
   </si>
   <si>
     <t>TC_141</t>
@@ -235,7 +235,7 @@
     <t>Chat interface test 141</t>
   </si>
   <si>
-    <t>2026-08-11T05:17:49.766Z</t>
+    <t>2026-08-11T05:24:02.897Z</t>
   </si>
   <si>
     <t>TC_142</t>
@@ -244,7 +244,7 @@
     <t>Chat interface test 142</t>
   </si>
   <si>
-    <t>2026-08-11T05:18:00.953Z</t>
+    <t>2026-08-11T05:24:08.480Z</t>
   </si>
   <si>
     <t>TC_143</t>
@@ -253,7 +253,7 @@
     <t>Chat interface test 143</t>
   </si>
   <si>
-    <t>2026-08-11T05:18:12.275Z</t>
+    <t>2026-08-11T05:24:13.755Z</t>
   </si>
   <si>
     <t>TC_144</t>
@@ -262,7 +262,7 @@
     <t>Chat interface test 144</t>
   </si>
   <si>
-    <t>2026-08-11T05:18:21.590Z</t>
+    <t>2026-08-11T05:24:19.147Z</t>
   </si>
   <si>
     <t>TC_145</t>
@@ -271,7 +271,7 @@
     <t>Chat interface test 145</t>
   </si>
   <si>
-    <t>2026-08-11T05:18:31.280Z</t>
+    <t>2026-08-11T05:24:24.765Z</t>
   </si>
   <si>
     <t>TC_146</t>
@@ -280,7 +280,7 @@
     <t>Chat interface test 146</t>
   </si>
   <si>
-    <t>2026-08-11T05:18:36.533Z</t>
+    <t>2026-08-11T05:24:30.127Z</t>
   </si>
   <si>
     <t>TC_147</t>
@@ -289,7 +289,7 @@
     <t>Chat interface test 147</t>
   </si>
   <si>
-    <t>2026-08-11T05:18:40.986Z</t>
+    <t>2026-08-11T05:24:36.011Z</t>
   </si>
   <si>
     <t>TC_148</t>
@@ -298,7 +298,7 @@
     <t>Chat interface test 148</t>
   </si>
   <si>
-    <t>2026-08-11T05:18:46.016Z</t>
+    <t>2026-08-11T05:24:42.464Z</t>
   </si>
   <si>
     <t>TC_149</t>
@@ -307,7 +307,7 @@
     <t>Chat interface test 149</t>
   </si>
   <si>
-    <t>2026-08-11T05:18:50.266Z</t>
+    <t>2026-08-11T05:24:48.494Z</t>
   </si>
   <si>
     <t>TC_150</t>
@@ -316,7 +316,7 @@
     <t>Chat interface test 150</t>
   </si>
   <si>
-    <t>2026-08-11T05:18:54.533Z</t>
+    <t>2026-08-11T05:24:54.168Z</t>
   </si>
   <si>
     <t>TC_151</t>
@@ -325,7 +325,7 @@
     <t>Chat interface test 151</t>
   </si>
   <si>
-    <t>2026-08-11T05:18:58.923Z</t>
+    <t>2026-08-11T05:25:02.089Z</t>
   </si>
   <si>
     <t>TC_152</t>
@@ -334,7 +334,7 @@
     <t>Chat interface test 152</t>
   </si>
   <si>
-    <t>2026-08-11T05:19:03.483Z</t>
+    <t>2026-08-11T05:25:08.066Z</t>
   </si>
   <si>
     <t>TC_153</t>
@@ -343,7 +343,7 @@
     <t>Chat interface test 153</t>
   </si>
   <si>
-    <t>2026-08-11T05:19:07.912Z</t>
+    <t>2026-08-11T05:25:13.265Z</t>
   </si>
   <si>
     <t>TC_154</t>
@@ -352,7 +352,7 @@
     <t>Chat interface test 154</t>
   </si>
   <si>
-    <t>2026-08-11T05:19:12.428Z</t>
+    <t>2026-08-11T05:25:18.622Z</t>
   </si>
   <si>
     <t>TC_155</t>
@@ -361,7 +361,7 @@
     <t>Chat interface test 155</t>
   </si>
   <si>
-    <t>2026-08-11T05:19:16.658Z</t>
+    <t>2026-08-11T05:25:23.790Z</t>
   </si>
   <si>
     <t>TC_156</t>
@@ -373,7 +373,7 @@
     <t>Notifications</t>
   </si>
   <si>
-    <t>2026-08-11T05:19:21.003Z</t>
+    <t>2026-08-11T05:25:28.675Z</t>
   </si>
   <si>
     <t>TC_157</t>
@@ -382,7 +382,7 @@
     <t>Notifications test 157</t>
   </si>
   <si>
-    <t>2026-08-11T05:19:25.209Z</t>
+    <t>2026-08-11T05:25:33.609Z</t>
   </si>
   <si>
     <t>TC_158</t>
@@ -391,7 +391,7 @@
     <t>Notifications test 158</t>
   </si>
   <si>
-    <t>2026-08-11T05:19:29.788Z</t>
+    <t>2026-08-11T05:25:38.132Z</t>
   </si>
   <si>
     <t>TC_159</t>
@@ -400,7 +400,7 @@
     <t>Notifications test 159</t>
   </si>
   <si>
-    <t>2026-08-11T05:19:33.924Z</t>
+    <t>2026-08-11T05:25:43.137Z</t>
   </si>
   <si>
     <t>TC_160</t>
@@ -409,7 +409,7 @@
     <t>Notifications test 160</t>
   </si>
   <si>
-    <t>2026-08-11T05:19:38.676Z</t>
+    <t>2026-08-11T05:25:47.694Z</t>
   </si>
   <si>
     <t>TC_161</t>
@@ -418,7 +418,7 @@
     <t>Notifications test 161</t>
   </si>
   <si>
-    <t>2026-08-11T05:19:43.813Z</t>
+    <t>2026-08-11T05:25:52.116Z</t>
   </si>
   <si>
     <t>TC_162</t>
@@ -427,7 +427,7 @@
     <t>Notifications test 162</t>
   </si>
   <si>
-    <t>2026-08-11T05:19:48.660Z</t>
+    <t>2026-08-11T05:25:57.007Z</t>
   </si>
   <si>
     <t>TC_163</t>
@@ -436,7 +436,7 @@
     <t>Notifications test 163</t>
   </si>
   <si>
-    <t>2026-08-11T05:19:53.929Z</t>
+    <t>2026-08-11T05:26:01.619Z</t>
   </si>
   <si>
     <t>TC_164</t>
@@ -445,7 +445,7 @@
     <t>Notifications test 164</t>
   </si>
   <si>
-    <t>2026-08-11T05:19:59.192Z</t>
+    <t>2026-08-11T05:26:06.969Z</t>
   </si>
   <si>
     <t>TC_165</t>
@@ -454,7 +454,7 @@
     <t>Notifications test 165</t>
   </si>
   <si>
-    <t>2026-08-11T05:20:03.415Z</t>
+    <t>2026-08-11T05:26:11.501Z</t>
   </si>
   <si>
     <t>TC_166</t>
@@ -463,7 +463,7 @@
     <t>Notifications test 166</t>
   </si>
   <si>
-    <t>2026-08-11T05:20:07.928Z</t>
+    <t>2026-08-11T05:26:17.129Z</t>
   </si>
   <si>
     <t>TC_167</t>
@@ -472,7 +472,7 @@
     <t>Notifications test 167</t>
   </si>
   <si>
-    <t>2026-08-11T05:20:12.399Z</t>
+    <t>2026-08-11T05:26:22.703Z</t>
   </si>
   <si>
     <t>TC_168</t>
@@ -481,7 +481,7 @@
     <t>Notifications test 168</t>
   </si>
   <si>
-    <t>2026-08-11T05:20:16.513Z</t>
+    <t>2026-08-11T05:26:27.389Z</t>
   </si>
   <si>
     <t>TC_169</t>
@@ -490,7 +490,7 @@
     <t>Notifications test 169</t>
   </si>
   <si>
-    <t>2026-08-11T05:20:21.568Z</t>
+    <t>2026-08-11T05:26:31.725Z</t>
   </si>
   <si>
     <t>TC_170</t>
@@ -499,7 +499,7 @@
     <t>Notifications test 170</t>
   </si>
   <si>
-    <t>2026-08-11T05:20:28.210Z</t>
+    <t>2026-08-11T05:26:35.850Z</t>
   </si>
   <si>
     <t>TC_171</t>
@@ -508,7 +508,7 @@
     <t>Notifications test 171</t>
   </si>
   <si>
-    <t>2026-08-11T05:20:33.690Z</t>
+    <t>2026-08-11T05:26:40.230Z</t>
   </si>
   <si>
     <t>TC_172</t>
@@ -517,7 +517,7 @@
     <t>Notifications test 172</t>
   </si>
   <si>
-    <t>2026-08-11T05:20:41.787Z</t>
+    <t>2026-08-11T05:26:44.849Z</t>
   </si>
   <si>
     <t>TC_173</t>
@@ -526,7 +526,7 @@
     <t>Notifications test 173</t>
   </si>
   <si>
-    <t>2026-08-11T05:20:46.626Z</t>
+    <t>2026-08-11T05:26:49.571Z</t>
   </si>
   <si>
     <t>TC_174</t>
@@ -535,7 +535,7 @@
     <t>Notifications test 174</t>
   </si>
   <si>
-    <t>2026-08-11T05:20:51.274Z</t>
+    <t>2026-08-11T05:26:54.136Z</t>
   </si>
   <si>
     <t>TC_175</t>
@@ -544,7 +544,7 @@
     <t>Notifications test 175</t>
   </si>
   <si>
-    <t>2026-08-11T05:20:55.806Z</t>
+    <t>2026-08-11T05:26:58.610Z</t>
   </si>
   <si>
     <t>TC_176</t>
@@ -553,7 +553,7 @@
     <t>Notifications test 176</t>
   </si>
   <si>
-    <t>2026-08-11T05:21:00.596Z</t>
+    <t>2026-08-11T05:27:03.100Z</t>
   </si>
   <si>
     <t>TC_177</t>
@@ -562,7 +562,7 @@
     <t>Notifications test 177</t>
   </si>
   <si>
-    <t>2026-08-11T05:21:05.068Z</t>
+    <t>2026-08-11T05:27:07.466Z</t>
   </si>
   <si>
     <t>TC_178</t>
@@ -571,7 +571,7 @@
     <t>Notifications test 178</t>
   </si>
   <si>
-    <t>2026-08-11T05:21:09.689Z</t>
+    <t>2026-08-11T05:27:13.170Z</t>
   </si>
   <si>
     <t>TC_179</t>
@@ -580,7 +580,7 @@
     <t>Notifications test 179</t>
   </si>
   <si>
-    <t>2026-08-11T05:21:14.629Z</t>
+    <t>2026-08-11T05:27:17.536Z</t>
   </si>
   <si>
     <t>TC_180</t>
@@ -589,7 +589,7 @@
     <t>Notifications test 180</t>
   </si>
   <si>
-    <t>2026-08-11T05:21:20.857Z</t>
+    <t>2026-08-11T05:27:21.672Z</t>
   </si>
 </sst>
 </file>
@@ -1042,7 +1042,7 @@
         <v>12</v>
       </c>
       <c r="F2">
-        <v>11757</v>
+        <v>6584</v>
       </c>
       <c r="G2" t="s">
         <v>13</v>
@@ -1068,7 +1068,7 @@
         <v>12</v>
       </c>
       <c r="F3">
-        <v>11721</v>
+        <v>6825</v>
       </c>
       <c r="G3" t="s">
         <v>16</v>
@@ -1094,7 +1094,7 @@
         <v>12</v>
       </c>
       <c r="F4">
-        <v>12089</v>
+        <v>6671</v>
       </c>
       <c r="G4" t="s">
         <v>19</v>
@@ -1120,7 +1120,7 @@
         <v>12</v>
       </c>
       <c r="F5">
-        <v>9868</v>
+        <v>6287</v>
       </c>
       <c r="G5" t="s">
         <v>22</v>
@@ -1146,7 +1146,7 @@
         <v>12</v>
       </c>
       <c r="F6">
-        <v>7679</v>
+        <v>8468</v>
       </c>
       <c r="G6" t="s">
         <v>25</v>
@@ -1172,7 +1172,7 @@
         <v>12</v>
       </c>
       <c r="F7">
-        <v>10153</v>
+        <v>8999</v>
       </c>
       <c r="G7" t="s">
         <v>28</v>
@@ -1198,7 +1198,7 @@
         <v>12</v>
       </c>
       <c r="F8">
-        <v>7861</v>
+        <v>9506</v>
       </c>
       <c r="G8" t="s">
         <v>31</v>
@@ -1224,7 +1224,7 @@
         <v>12</v>
       </c>
       <c r="F9">
-        <v>8640</v>
+        <v>7842</v>
       </c>
       <c r="G9" t="s">
         <v>34</v>
@@ -1250,7 +1250,7 @@
         <v>12</v>
       </c>
       <c r="F10">
-        <v>8644</v>
+        <v>5903</v>
       </c>
       <c r="G10" t="s">
         <v>37</v>
@@ -1276,7 +1276,7 @@
         <v>12</v>
       </c>
       <c r="F11">
-        <v>10409</v>
+        <v>8779</v>
       </c>
       <c r="G11" t="s">
         <v>40</v>
@@ -1302,7 +1302,7 @@
         <v>12</v>
       </c>
       <c r="F12">
-        <v>9217</v>
+        <v>10283</v>
       </c>
       <c r="G12" t="s">
         <v>43</v>
@@ -1328,7 +1328,7 @@
         <v>12</v>
       </c>
       <c r="F13">
-        <v>9984</v>
+        <v>7851</v>
       </c>
       <c r="G13" t="s">
         <v>46</v>
@@ -1354,7 +1354,7 @@
         <v>12</v>
       </c>
       <c r="F14">
-        <v>7523</v>
+        <v>12514</v>
       </c>
       <c r="G14" t="s">
         <v>49</v>
@@ -1380,7 +1380,7 @@
         <v>12</v>
       </c>
       <c r="F15">
-        <v>9850</v>
+        <v>7106</v>
       </c>
       <c r="G15" t="s">
         <v>52</v>
@@ -1406,7 +1406,7 @@
         <v>12</v>
       </c>
       <c r="F16">
-        <v>10409</v>
+        <v>6300</v>
       </c>
       <c r="G16" t="s">
         <v>55</v>
@@ -1432,7 +1432,7 @@
         <v>12</v>
       </c>
       <c r="F17">
-        <v>11269</v>
+        <v>7466</v>
       </c>
       <c r="G17" t="s">
         <v>59</v>
@@ -1458,7 +1458,7 @@
         <v>12</v>
       </c>
       <c r="F18">
-        <v>10766</v>
+        <v>5631</v>
       </c>
       <c r="G18" t="s">
         <v>62</v>
@@ -1484,7 +1484,7 @@
         <v>12</v>
       </c>
       <c r="F19">
-        <v>10798</v>
+        <v>5378</v>
       </c>
       <c r="G19" t="s">
         <v>65</v>
@@ -1510,7 +1510,7 @@
         <v>12</v>
       </c>
       <c r="F20">
-        <v>12850</v>
+        <v>5588</v>
       </c>
       <c r="G20" t="s">
         <v>68</v>
@@ -1536,7 +1536,7 @@
         <v>12</v>
       </c>
       <c r="F21">
-        <v>10676</v>
+        <v>6026</v>
       </c>
       <c r="G21" t="s">
         <v>71</v>
@@ -1562,7 +1562,7 @@
         <v>12</v>
       </c>
       <c r="F22">
-        <v>12581</v>
+        <v>4966</v>
       </c>
       <c r="G22" t="s">
         <v>74</v>
@@ -1588,7 +1588,7 @@
         <v>12</v>
       </c>
       <c r="F23">
-        <v>11181</v>
+        <v>5581</v>
       </c>
       <c r="G23" t="s">
         <v>77</v>
@@ -1614,7 +1614,7 @@
         <v>12</v>
       </c>
       <c r="F24">
-        <v>11310</v>
+        <v>5272</v>
       </c>
       <c r="G24" t="s">
         <v>80</v>
@@ -1640,7 +1640,7 @@
         <v>12</v>
       </c>
       <c r="F25">
-        <v>9300</v>
+        <v>5391</v>
       </c>
       <c r="G25" t="s">
         <v>83</v>
@@ -1666,7 +1666,7 @@
         <v>12</v>
       </c>
       <c r="F26">
-        <v>9684</v>
+        <v>5617</v>
       </c>
       <c r="G26" t="s">
         <v>86</v>
@@ -1692,7 +1692,7 @@
         <v>12</v>
       </c>
       <c r="F27">
-        <v>5251</v>
+        <v>5360</v>
       </c>
       <c r="G27" t="s">
         <v>89</v>
@@ -1718,7 +1718,7 @@
         <v>12</v>
       </c>
       <c r="F28">
-        <v>4451</v>
+        <v>5883</v>
       </c>
       <c r="G28" t="s">
         <v>92</v>
@@ -1744,7 +1744,7 @@
         <v>12</v>
       </c>
       <c r="F29">
-        <v>5029</v>
+        <v>6451</v>
       </c>
       <c r="G29" t="s">
         <v>95</v>
@@ -1770,7 +1770,7 @@
         <v>12</v>
       </c>
       <c r="F30">
-        <v>4249</v>
+        <v>6028</v>
       </c>
       <c r="G30" t="s">
         <v>98</v>
@@ -1796,7 +1796,7 @@
         <v>12</v>
       </c>
       <c r="F31">
-        <v>4266</v>
+        <v>5673</v>
       </c>
       <c r="G31" t="s">
         <v>101</v>
@@ -1822,7 +1822,7 @@
         <v>12</v>
       </c>
       <c r="F32">
-        <v>4388</v>
+        <v>7919</v>
       </c>
       <c r="G32" t="s">
         <v>104</v>
@@ -1848,7 +1848,7 @@
         <v>12</v>
       </c>
       <c r="F33">
-        <v>4559</v>
+        <v>5974</v>
       </c>
       <c r="G33" t="s">
         <v>107</v>
@@ -1874,7 +1874,7 @@
         <v>12</v>
       </c>
       <c r="F34">
-        <v>4428</v>
+        <v>5197</v>
       </c>
       <c r="G34" t="s">
         <v>110</v>
@@ -1900,7 +1900,7 @@
         <v>12</v>
       </c>
       <c r="F35">
-        <v>4515</v>
+        <v>5355</v>
       </c>
       <c r="G35" t="s">
         <v>113</v>
@@ -1926,7 +1926,7 @@
         <v>12</v>
       </c>
       <c r="F36">
-        <v>4228</v>
+        <v>5166</v>
       </c>
       <c r="G36" t="s">
         <v>116</v>
@@ -1952,7 +1952,7 @@
         <v>12</v>
       </c>
       <c r="F37">
-        <v>4344</v>
+        <v>4883</v>
       </c>
       <c r="G37" t="s">
         <v>120</v>
@@ -1978,7 +1978,7 @@
         <v>12</v>
       </c>
       <c r="F38">
-        <v>4205</v>
+        <v>4932</v>
       </c>
       <c r="G38" t="s">
         <v>123</v>
@@ -2004,7 +2004,7 @@
         <v>12</v>
       </c>
       <c r="F39">
-        <v>4577</v>
+        <v>4521</v>
       </c>
       <c r="G39" t="s">
         <v>126</v>
@@ -2030,7 +2030,7 @@
         <v>12</v>
       </c>
       <c r="F40">
-        <v>4135</v>
+        <v>5003</v>
       </c>
       <c r="G40" t="s">
         <v>129</v>
@@ -2056,7 +2056,7 @@
         <v>12</v>
       </c>
       <c r="F41">
-        <v>4751</v>
+        <v>4556</v>
       </c>
       <c r="G41" t="s">
         <v>132</v>
@@ -2082,7 +2082,7 @@
         <v>12</v>
       </c>
       <c r="F42">
-        <v>5136</v>
+        <v>4420</v>
       </c>
       <c r="G42" t="s">
         <v>135</v>
@@ -2108,7 +2108,7 @@
         <v>12</v>
       </c>
       <c r="F43">
-        <v>4846</v>
+        <v>4890</v>
       </c>
       <c r="G43" t="s">
         <v>138</v>
@@ -2134,7 +2134,7 @@
         <v>12</v>
       </c>
       <c r="F44">
-        <v>5268</v>
+        <v>4611</v>
       </c>
       <c r="G44" t="s">
         <v>141</v>
@@ -2160,7 +2160,7 @@
         <v>12</v>
       </c>
       <c r="F45">
-        <v>5261</v>
+        <v>5348</v>
       </c>
       <c r="G45" t="s">
         <v>144</v>
@@ -2186,7 +2186,7 @@
         <v>12</v>
       </c>
       <c r="F46">
-        <v>4222</v>
+        <v>4529</v>
       </c>
       <c r="G46" t="s">
         <v>147</v>
@@ -2212,7 +2212,7 @@
         <v>12</v>
       </c>
       <c r="F47">
-        <v>4512</v>
+        <v>5625</v>
       </c>
       <c r="G47" t="s">
         <v>150</v>
@@ -2238,7 +2238,7 @@
         <v>12</v>
       </c>
       <c r="F48">
-        <v>4470</v>
+        <v>5572</v>
       </c>
       <c r="G48" t="s">
         <v>153</v>
@@ -2264,7 +2264,7 @@
         <v>12</v>
       </c>
       <c r="F49">
-        <v>4112</v>
+        <v>4684</v>
       </c>
       <c r="G49" t="s">
         <v>156</v>
@@ -2290,7 +2290,7 @@
         <v>12</v>
       </c>
       <c r="F50">
-        <v>5054</v>
+        <v>4335</v>
       </c>
       <c r="G50" t="s">
         <v>159</v>
@@ -2316,7 +2316,7 @@
         <v>12</v>
       </c>
       <c r="F51">
-        <v>6640</v>
+        <v>4124</v>
       </c>
       <c r="G51" t="s">
         <v>162</v>
@@ -2342,7 +2342,7 @@
         <v>12</v>
       </c>
       <c r="F52">
-        <v>5478</v>
+        <v>4377</v>
       </c>
       <c r="G52" t="s">
         <v>165</v>
@@ -2368,7 +2368,7 @@
         <v>12</v>
       </c>
       <c r="F53">
-        <v>8096</v>
+        <v>4617</v>
       </c>
       <c r="G53" t="s">
         <v>168</v>
@@ -2394,7 +2394,7 @@
         <v>12</v>
       </c>
       <c r="F54">
-        <v>4838</v>
+        <v>4720</v>
       </c>
       <c r="G54" t="s">
         <v>171</v>
@@ -2420,7 +2420,7 @@
         <v>12</v>
       </c>
       <c r="F55">
-        <v>4647</v>
+        <v>4564</v>
       </c>
       <c r="G55" t="s">
         <v>174</v>
@@ -2446,7 +2446,7 @@
         <v>12</v>
       </c>
       <c r="F56">
-        <v>4530</v>
+        <v>4473</v>
       </c>
       <c r="G56" t="s">
         <v>177</v>
@@ -2472,7 +2472,7 @@
         <v>12</v>
       </c>
       <c r="F57">
-        <v>4789</v>
+        <v>4488</v>
       </c>
       <c r="G57" t="s">
         <v>180</v>
@@ -2498,7 +2498,7 @@
         <v>12</v>
       </c>
       <c r="F58">
-        <v>4471</v>
+        <v>4365</v>
       </c>
       <c r="G58" t="s">
         <v>183</v>
@@ -2524,7 +2524,7 @@
         <v>12</v>
       </c>
       <c r="F59">
-        <v>4620</v>
+        <v>5702</v>
       </c>
       <c r="G59" t="s">
         <v>186</v>
@@ -2550,7 +2550,7 @@
         <v>12</v>
       </c>
       <c r="F60">
-        <v>4938</v>
+        <v>4365</v>
       </c>
       <c r="G60" t="s">
         <v>189</v>
@@ -2576,7 +2576,7 @@
         <v>12</v>
       </c>
       <c r="F61">
-        <v>6227</v>
+        <v>4135</v>
       </c>
       <c r="G61" t="s">
         <v>192</v>

</xml_diff>